<commit_message>
Update analysis to nested CES and publish current results
</commit_message>
<xml_diff>
--- a/5_simulation/outputs/tables/supplementary/S12_micro_sensitivity.xlsx
+++ b/5_simulation/outputs/tables/supplementary/S12_micro_sensitivity.xlsx
@@ -497,34 +497,34 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15.9903354494</v>
+        <v>16.0168009360714</v>
       </c>
       <c r="E2" t="n">
-        <v>4.73467731473</v>
+        <v>4.739008249705113</v>
       </c>
       <c r="F2" t="n">
-        <v>2.03089194576</v>
+        <v>2.032888313228137</v>
       </c>
       <c r="G2" t="n">
-        <v>2.26188565834</v>
+        <v>2.229091928501387</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.893612349065</v>
+        <v>-0.9203494029995636</v>
       </c>
       <c r="I2" t="n">
-        <v>5.39346755406</v>
+        <v>5.70700918541707</v>
       </c>
       <c r="J2" t="n">
-        <v>0.168718799193</v>
+        <v>0.2094720644353072</v>
       </c>
       <c r="K2" t="n">
-        <v>1.7763568394e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.394764010794</v>
+        <v>0.3947878001027232</v>
       </c>
     </row>
     <row r="3">
@@ -540,34 +540,34 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16.2309434674</v>
+        <v>16.26367665466252</v>
       </c>
       <c r="E3" t="n">
-        <v>4.8084763814</v>
+        <v>4.812829062167006</v>
       </c>
       <c r="F3" t="n">
-        <v>2.06426193151</v>
+        <v>2.066288126971348</v>
       </c>
       <c r="G3" t="n">
-        <v>1.10976247066</v>
+        <v>1.077504418528695</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.8932020649770001</v>
+        <v>-0.9199436667357968</v>
       </c>
       <c r="I3" t="n">
-        <v>29.9466907135</v>
+        <v>30.06239298366212</v>
       </c>
       <c r="J3" t="n">
-        <v>0.177636894028</v>
+        <v>0.1748805127934855</v>
       </c>
       <c r="K3" t="n">
-        <v>1.55431223448e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.395792151785</v>
+        <v>0.3958154625442059</v>
       </c>
     </row>
     <row r="4">
@@ -583,34 +583,34 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>16.8340567199</v>
+        <v>16.83405671989201</v>
       </c>
       <c r="E4" t="n">
-        <v>5.15895544941</v>
+        <v>5.163423298266742</v>
       </c>
       <c r="F4" t="n">
-        <v>2.29045335473</v>
+        <v>2.292567737378171</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.250257235465</v>
+        <v>-0.2817783294058053</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.890668060596</v>
+        <v>-0.9174248743812805</v>
       </c>
       <c r="I4" t="n">
-        <v>47.2118384312</v>
+        <v>48.17026952202748</v>
       </c>
       <c r="J4" t="n">
-        <v>0.146145315866</v>
+        <v>0.1273996634505085</v>
       </c>
       <c r="K4" t="n">
-        <v>2.22044604925e-15</v>
+        <v>1.77635683940025e-15</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.398637349043</v>
+        <v>0.3986603568106426</v>
       </c>
     </row>
     <row r="5">
@@ -626,34 +626,34 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>16.8280212787</v>
+        <v>16.82802127866404</v>
       </c>
       <c r="E5" t="n">
-        <v>5.27086771487</v>
+        <v>5.272314250064657</v>
       </c>
       <c r="F5" t="n">
-        <v>2.38232555199</v>
+        <v>2.383045979641087</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.703091646905</v>
+        <v>-0.7160148336489793</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.881111257089</v>
+        <v>-0.893054988761786</v>
       </c>
       <c r="I5" t="n">
-        <v>85.024899408</v>
+        <v>85.79907123733406</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0951022213208</v>
+        <v>0.1663486893538007</v>
       </c>
       <c r="K5" t="n">
-        <v>1.11022302463e-15</v>
+        <v>8.881784197001252e-16</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.399942424002</v>
+        <v>0.399941048335793</v>
       </c>
     </row>
     <row r="6">
@@ -669,34 +669,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16.027627399</v>
+        <v>16.03425538486147</v>
       </c>
       <c r="E6" t="n">
-        <v>4.72111737875</v>
+        <v>4.725313265298551</v>
       </c>
       <c r="F6" t="n">
-        <v>2.02356783159</v>
+        <v>2.02550929816374</v>
       </c>
       <c r="G6" t="n">
-        <v>2.26488523824</v>
+        <v>2.23170326253087</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.894526278968</v>
+        <v>-0.9218203659532466</v>
       </c>
       <c r="I6" t="n">
-        <v>5.92809487654</v>
+        <v>6.146084882494511</v>
       </c>
       <c r="J6" t="n">
-        <v>1.00325059531e-13</v>
+        <v>1.042701902634174e-13</v>
       </c>
       <c r="K6" t="n">
-        <v>1.7763568394e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0.394731272159</v>
+        <v>0.3947569121972629</v>
       </c>
     </row>
     <row r="7">
@@ -712,34 +712,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16.2686554943</v>
+        <v>16.27868675027158</v>
       </c>
       <c r="E7" t="n">
-        <v>4.79512145664</v>
+        <v>4.799340773615971</v>
       </c>
       <c r="F7" t="n">
-        <v>2.05687440786</v>
+        <v>2.058841325942624</v>
       </c>
       <c r="G7" t="n">
-        <v>1.11228779569</v>
+        <v>1.079623529294268</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.893660546124</v>
+        <v>-0.9209576215190235</v>
       </c>
       <c r="I7" t="n">
-        <v>30.1538207375</v>
+        <v>30.24489616661757</v>
       </c>
       <c r="J7" t="n">
-        <v>1.06974547682e-13</v>
+        <v>1.11291038665817e-13</v>
       </c>
       <c r="K7" t="n">
-        <v>1.55431223448e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>0.395761201461</v>
+        <v>0.3957863504182297</v>
       </c>
     </row>
     <row r="8">
@@ -755,34 +755,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>16.804541989</v>
+        <v>16.81221946945899</v>
       </c>
       <c r="E8" t="n">
-        <v>5.1455772468</v>
+        <v>5.149871065138074</v>
       </c>
       <c r="F8" t="n">
-        <v>2.28287335268</v>
+        <v>2.284928512343573</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.24995182567</v>
+        <v>-0.2818840539577651</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.891507501749</v>
+        <v>-0.9188123229556457</v>
       </c>
       <c r="I8" t="n">
-        <v>45.5677747649</v>
+        <v>46.42260079640627</v>
       </c>
       <c r="J8" t="n">
-        <v>8.412711547839999e-14</v>
+        <v>9.141398779233055e-14</v>
       </c>
       <c r="K8" t="n">
-        <v>2.22044604925e-15</v>
+        <v>1.77635683940025e-15</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.398605115368</v>
+        <v>0.3986299433876126</v>
       </c>
     </row>
     <row r="9">
@@ -798,34 +798,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>16.8813006953</v>
+        <v>16.88456649010951</v>
       </c>
       <c r="E9" t="n">
-        <v>5.27702081369</v>
+        <v>5.278362984948579</v>
       </c>
       <c r="F9" t="n">
-        <v>2.38754542325</v>
+        <v>2.388232568702799</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.704513167011</v>
+        <v>-0.7174836172690885</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.883173031914</v>
+        <v>-0.8954501315113115</v>
       </c>
       <c r="I9" t="n">
-        <v>93.25855283910001</v>
+        <v>94.21647941190787</v>
       </c>
       <c r="J9" t="n">
-        <v>9.018785270259999e-14</v>
+        <v>1.081743949451875e-13</v>
       </c>
       <c r="K9" t="n">
-        <v>1.11022302463e-15</v>
+        <v>8.881784197001252e-16</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>0.399999153613</v>
+        <v>0.3999985801583614</v>
       </c>
     </row>
     <row r="10">
@@ -841,34 +841,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>23.557174764</v>
+        <v>23.57882188384849</v>
       </c>
       <c r="E10" t="n">
-        <v>7.21456921369</v>
+        <v>7.220856983793082</v>
       </c>
       <c r="F10" t="n">
-        <v>3.23530618598</v>
+        <v>3.238309712598473</v>
       </c>
       <c r="G10" t="n">
-        <v>2.26188565834</v>
+        <v>2.229091928501387</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.893612349065</v>
+        <v>-0.9203494029995636</v>
       </c>
       <c r="I10" t="n">
-        <v>5.39346755406</v>
+        <v>5.70700918541707</v>
       </c>
       <c r="J10" t="n">
-        <v>0.168718799193</v>
+        <v>0.2094720644353072</v>
       </c>
       <c r="K10" t="n">
-        <v>1.7763568394e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>0.394764010794</v>
+        <v>0.3947878001027232</v>
       </c>
     </row>
     <row r="11">
@@ -884,34 +884,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24.0517869305</v>
+        <v>24.08555266842837</v>
       </c>
       <c r="E11" t="n">
-        <v>7.33756984026</v>
+        <v>7.343969389567907</v>
       </c>
       <c r="F11" t="n">
-        <v>3.28864919414</v>
+        <v>3.291691430555442</v>
       </c>
       <c r="G11" t="n">
-        <v>1.10976247066</v>
+        <v>1.077504418528695</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.8932020649770001</v>
+        <v>-0.9199436667357968</v>
       </c>
       <c r="I11" t="n">
-        <v>29.9466907135</v>
+        <v>30.06239298366212</v>
       </c>
       <c r="J11" t="n">
-        <v>0.177636894028</v>
+        <v>0.1748805127934855</v>
       </c>
       <c r="K11" t="n">
-        <v>1.55431223448e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.395792151785</v>
+        <v>0.3958154625442059</v>
       </c>
     </row>
     <row r="12">
@@ -927,34 +927,34 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>24.4413624382</v>
+        <v>24.45347239312542</v>
       </c>
       <c r="E12" t="n">
-        <v>7.72523275207</v>
+        <v>7.731657538654853</v>
       </c>
       <c r="F12" t="n">
-        <v>3.55872365005</v>
+        <v>3.561854017177356</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.250257235465</v>
+        <v>-0.2817783294058053</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.890668060596</v>
+        <v>-0.9174248743812805</v>
       </c>
       <c r="I12" t="n">
-        <v>47.2118384312</v>
+        <v>48.17026952202748</v>
       </c>
       <c r="J12" t="n">
-        <v>0.146145315866</v>
+        <v>0.1273996634505085</v>
       </c>
       <c r="K12" t="n">
-        <v>2.22044604925e-15</v>
+        <v>1.77635683940025e-15</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.398637349043</v>
+        <v>0.3986603568106426</v>
       </c>
     </row>
     <row r="13">
@@ -970,34 +970,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>24.4759450361</v>
+        <v>24.4759450360823</v>
       </c>
       <c r="E13" t="n">
-        <v>7.83381662796</v>
+        <v>7.835895213132503</v>
       </c>
       <c r="F13" t="n">
-        <v>3.65638387092</v>
+        <v>3.657417658007697</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.703091646905</v>
+        <v>-0.7160148336489793</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.881111257089</v>
+        <v>-0.893054988761786</v>
       </c>
       <c r="I13" t="n">
-        <v>85.024899408</v>
+        <v>85.79907123733406</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0951022213208</v>
+        <v>0.1663486893538007</v>
       </c>
       <c r="K13" t="n">
-        <v>1.11022302463e-15</v>
+        <v>8.881784197001252e-16</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>0.399942424002</v>
+        <v>0.399941048335793</v>
       </c>
     </row>
     <row r="14">
@@ -1013,34 +1013,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>23.4971471002</v>
+        <v>23.50294003232646</v>
       </c>
       <c r="E14" t="n">
-        <v>7.19675742901</v>
+        <v>7.202814295950992</v>
       </c>
       <c r="F14" t="n">
-        <v>3.2257529507</v>
+        <v>3.228670653055677</v>
       </c>
       <c r="G14" t="n">
-        <v>2.26488523824</v>
+        <v>2.23170326253087</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.894526278968</v>
+        <v>-0.9218203659532466</v>
       </c>
       <c r="I14" t="n">
-        <v>5.92809487654</v>
+        <v>6.146084882494511</v>
       </c>
       <c r="J14" t="n">
-        <v>1.00325059531e-13</v>
+        <v>1.042701902634174e-13</v>
       </c>
       <c r="K14" t="n">
-        <v>1.7763568394e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0.394731272159</v>
+        <v>0.3947569121972629</v>
       </c>
     </row>
     <row r="15">
@@ -1056,34 +1056,34 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>24.0060533953</v>
+        <v>24.00606872572989</v>
       </c>
       <c r="E15" t="n">
-        <v>7.31959225681</v>
+        <v>7.325749358932454</v>
       </c>
       <c r="F15" t="n">
-        <v>3.27899774185</v>
+        <v>3.281950399133893</v>
       </c>
       <c r="G15" t="n">
-        <v>1.11228779569</v>
+        <v>1.079623529294268</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.893660546124</v>
+        <v>-0.9209576215190235</v>
       </c>
       <c r="I15" t="n">
-        <v>30.1538207375</v>
+        <v>30.24489616661757</v>
       </c>
       <c r="J15" t="n">
-        <v>1.06974547682e-13</v>
+        <v>1.11291038665817e-13</v>
       </c>
       <c r="K15" t="n">
-        <v>1.55431223448e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0.395761201461</v>
+        <v>0.3957863504182297</v>
       </c>
     </row>
     <row r="16">
@@ -1099,34 +1099,34 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>24.4228131654</v>
+        <v>24.44275344717505</v>
       </c>
       <c r="E16" t="n">
-        <v>7.70734647737</v>
+        <v>7.713581738392182</v>
       </c>
       <c r="F16" t="n">
-        <v>3.54891901818</v>
+        <v>3.551959423945078</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.24995182567</v>
+        <v>-0.2818840539577651</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.891507501749</v>
+        <v>-0.9188123229556457</v>
       </c>
       <c r="I16" t="n">
-        <v>45.5677747649</v>
+        <v>46.42260079640627</v>
       </c>
       <c r="J16" t="n">
-        <v>8.412711547839999e-14</v>
+        <v>9.141398779233055e-14</v>
       </c>
       <c r="K16" t="n">
-        <v>2.22044604925e-15</v>
+        <v>1.77635683940025e-15</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>0.398605115368</v>
+        <v>0.3986299433876126</v>
       </c>
     </row>
     <row r="17">
@@ -1142,34 +1142,34 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>24.5609943403</v>
+        <v>24.5609943402641</v>
       </c>
       <c r="E17" t="n">
-        <v>7.83796337292</v>
+        <v>7.839895927328674</v>
       </c>
       <c r="F17" t="n">
-        <v>3.66147991624</v>
+        <v>3.662457199497565</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.704513167011</v>
+        <v>-0.7174836172690885</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.883173031914</v>
+        <v>-0.8954501315113115</v>
       </c>
       <c r="I17" t="n">
-        <v>93.25855283910001</v>
+        <v>94.21647941190787</v>
       </c>
       <c r="J17" t="n">
-        <v>9.018785270259999e-14</v>
+        <v>1.081743949451875e-13</v>
       </c>
       <c r="K17" t="n">
-        <v>1.11022302463e-15</v>
+        <v>8.881784197001252e-16</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>0.399999153613</v>
+        <v>0.3999985801583614</v>
       </c>
     </row>
     <row r="18">
@@ -1185,34 +1185,34 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>30.6369262701</v>
+        <v>30.63001006252545</v>
       </c>
       <c r="E18" t="n">
-        <v>10.043378823</v>
+        <v>10.05115642155338</v>
       </c>
       <c r="F18" t="n">
-        <v>4.67180235963</v>
+        <v>4.675877216260801</v>
       </c>
       <c r="G18" t="n">
-        <v>2.26188565834</v>
+        <v>2.229091928501387</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.893612349065</v>
+        <v>-0.9203494029995636</v>
       </c>
       <c r="I18" t="n">
-        <v>5.39346755406</v>
+        <v>5.70700918541707</v>
       </c>
       <c r="J18" t="n">
-        <v>0.168718799193</v>
+        <v>0.2094720644353072</v>
       </c>
       <c r="K18" t="n">
-        <v>1.7763568394e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>0.394764010794</v>
+        <v>0.3947878001027232</v>
       </c>
     </row>
     <row r="19">
@@ -1228,34 +1228,34 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>31.0450931594</v>
+        <v>31.05294688580065</v>
       </c>
       <c r="E19" t="n">
-        <v>10.2281169908</v>
+        <v>10.23593166687481</v>
       </c>
       <c r="F19" t="n">
-        <v>4.75286915304</v>
+        <v>4.756989632696062</v>
       </c>
       <c r="G19" t="n">
-        <v>1.10976247066</v>
+        <v>1.077504418528695</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.8932020649770001</v>
+        <v>-0.9199436667357968</v>
       </c>
       <c r="I19" t="n">
-        <v>29.9466907135</v>
+        <v>30.06239298366212</v>
       </c>
       <c r="J19" t="n">
-        <v>0.177636894028</v>
+        <v>0.1748805127934855</v>
       </c>
       <c r="K19" t="n">
-        <v>1.55431223448e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>0.395792151785</v>
+        <v>0.3958154625442059</v>
       </c>
     </row>
     <row r="20">
@@ -1271,34 +1271,34 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>31.1377473906</v>
+        <v>31.14145712128714</v>
       </c>
       <c r="E20" t="n">
-        <v>10.6011448807</v>
+        <v>10.60878642036503</v>
       </c>
       <c r="F20" t="n">
-        <v>5.05167917119</v>
+        <v>5.055857120807477</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.250257235465</v>
+        <v>-0.2817783294058053</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.890668060596</v>
+        <v>-0.9174248743812805</v>
       </c>
       <c r="I20" t="n">
-        <v>47.2118384312</v>
+        <v>48.17026952202748</v>
       </c>
       <c r="J20" t="n">
-        <v>0.146145315866</v>
+        <v>0.1273996634505085</v>
       </c>
       <c r="K20" t="n">
-        <v>2.22044604925e-15</v>
+        <v>1.77635683940025e-15</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>0.398637349043</v>
+        <v>0.3986603568106426</v>
       </c>
     </row>
     <row r="21">
@@ -1314,34 +1314,34 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31.1527926081</v>
+        <v>31.17653800374298</v>
       </c>
       <c r="E21" t="n">
-        <v>10.6919406608</v>
+        <v>10.69463678528712</v>
       </c>
       <c r="F21" t="n">
-        <v>5.15009141314</v>
+        <v>5.151482334041808</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.703091646905</v>
+        <v>-0.7160148336489793</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.881111257089</v>
+        <v>-0.893054988761786</v>
       </c>
       <c r="I21" t="n">
-        <v>85.024899408</v>
+        <v>85.79907123733406</v>
       </c>
       <c r="J21" t="n">
-        <v>0.0951022213208</v>
+        <v>0.1663486893538007</v>
       </c>
       <c r="K21" t="n">
-        <v>1.11022302463e-15</v>
+        <v>8.881784197001252e-16</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>0.399942424002</v>
+        <v>0.399941048335793</v>
       </c>
     </row>
     <row r="22">
@@ -1357,34 +1357,34 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>30.4233366709</v>
+        <v>30.45312360768395</v>
       </c>
       <c r="E22" t="n">
-        <v>10.0200603663</v>
+        <v>10.02746846531047</v>
       </c>
       <c r="F22" t="n">
-        <v>4.65959119979</v>
+        <v>4.663538339257022</v>
       </c>
       <c r="G22" t="n">
-        <v>2.26488523824</v>
+        <v>2.23170326253087</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.894526278968</v>
+        <v>-0.9218203659532466</v>
       </c>
       <c r="I22" t="n">
-        <v>5.92809487654</v>
+        <v>6.146084882494511</v>
       </c>
       <c r="J22" t="n">
-        <v>1.00325059531e-13</v>
+        <v>1.042701902634174e-13</v>
       </c>
       <c r="K22" t="n">
-        <v>1.7763568394e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>0.394731272159</v>
+        <v>0.3947569121972629</v>
       </c>
     </row>
     <row r="23">
@@ -1400,34 +1400,34 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>30.8408306638</v>
+        <v>30.89075546515817</v>
       </c>
       <c r="E23" t="n">
-        <v>10.204692336</v>
+        <v>10.21210040777291</v>
       </c>
       <c r="F23" t="n">
-        <v>4.74048894985</v>
+        <v>4.744477274143006</v>
       </c>
       <c r="G23" t="n">
-        <v>1.11228779569</v>
+        <v>1.079623529294268</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.893660546124</v>
+        <v>-0.9209576215190235</v>
       </c>
       <c r="I23" t="n">
-        <v>30.1538207375</v>
+        <v>30.24489616661757</v>
       </c>
       <c r="J23" t="n">
-        <v>1.06974547682e-13</v>
+        <v>1.11291038665817e-13</v>
       </c>
       <c r="K23" t="n">
-        <v>1.55431223448e-15</v>
+        <v>2.664535259100376e-15</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>0.395761201461</v>
+        <v>0.3957863504182297</v>
       </c>
     </row>
     <row r="24">
@@ -1443,34 +1443,34 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>31.1124615526</v>
+        <v>31.11445429461222</v>
       </c>
       <c r="E24" t="n">
-        <v>10.5778241476</v>
+        <v>10.58515872662438</v>
       </c>
       <c r="F24" t="n">
-        <v>5.03917092894</v>
+        <v>5.043215771149542</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.24995182567</v>
+        <v>-0.2818840539577651</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.891507501749</v>
+        <v>-0.9188123229556457</v>
       </c>
       <c r="I24" t="n">
-        <v>45.5677747649</v>
+        <v>46.42260079640627</v>
       </c>
       <c r="J24" t="n">
-        <v>8.412711547839999e-14</v>
+        <v>9.141398779233055e-14</v>
       </c>
       <c r="K24" t="n">
-        <v>2.22044604925e-15</v>
+        <v>1.77635683940025e-15</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>0.398605115368</v>
+        <v>0.3986299433876126</v>
       </c>
     </row>
     <row r="25">
@@ -1486,34 +1486,34 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>31.1505293836</v>
+        <v>31.15052938357521</v>
       </c>
       <c r="E25" t="n">
-        <v>10.6965411718</v>
+        <v>10.69899957513215</v>
       </c>
       <c r="F25" t="n">
-        <v>5.15507799115</v>
+        <v>5.15638013334104</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.704513167011</v>
+        <v>-0.7174836172690885</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.883173031914</v>
+        <v>-0.8954501315113115</v>
       </c>
       <c r="I25" t="n">
-        <v>93.25855283910001</v>
+        <v>94.21647941190787</v>
       </c>
       <c r="J25" t="n">
-        <v>9.018785270259999e-14</v>
+        <v>1.081743949451875e-13</v>
       </c>
       <c r="K25" t="n">
-        <v>1.11022302463e-15</v>
+        <v>8.881784197001252e-16</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>0.399999153613</v>
+        <v>0.3999985801583614</v>
       </c>
     </row>
   </sheetData>

</xml_diff>